<commit_message>
docs: reconcile VERIFICATION_PLAN_v2.md + test-plan xlsx with the 99.17% ISACOV result
VERIFICATION_PLAN_v2.md: superseded the frozen 2026-09-06 83.14% figure (row L1
history, C-ISA row, W-13 row) with the round-by-round history to 99.17%
(477/481, 99.57% weighted), the OBS-068/OBS-069 findings, and a pointer to the
new docs/riscvisacov/RISCVISACOV_INSTRUCTION_REFERENCE.md. Carried over the
same provenance-gap disclosure (2026-09-09's larger, now-unreproducible
1,812/6,929 measurement) already recorded in RISCVISACOV_STATUS.md.

Vortex_UVM_Verification_Test_Plan.xlsx: updated FC-10 (Feature Coverage sheet),
TP-18 (Test Plan sheet), and R-014 (Traceability Matrix sheet) with the current
477/481 = 99.17% figure and citations to OBS-068/OBS-069 and the new
instruction-reference doc; added a v1.1 Revision History row.
</commit_message>
<xml_diff>
--- a/docs/Vortex_UVM_Verification_Test_Plan.xlsx
+++ b/docs/Vortex_UVM_Verification_Test_Plan.xlsx
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H21" s="40" t="inlineStr">
         <is>
-          <t>78/80 covergroups real; 2 structurally dead (fence.i mis-decode, an unset-define-gated coverpoint)</t>
+          <t>477/481 covergroups real (99.17%, 99.57% weighted); 4 bins honestly open (2 deferred jalr imm, 2 unexplained CSR rd_sign); fence.i/nop permanently 0% by construction</t>
         </is>
       </c>
       <c r="I21" s="40" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="P21" s="40" t="inlineStr">
         <is>
-          <t>docs/RTL_OBSERVATIONS.md OBS-056</t>
+          <t>docs/RTL_OBSERVATIONS.md OBS-056, OBS-068, OBS-069; docs/riscvisacov/RISCVISACOV_INSTRUCTION_REFERENCE.md</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="C18" s="40" t="inlineStr">
         <is>
-          <t>docs/RTL_OBSERVATIONS.md OBS-056</t>
+          <t>docs/RTL_OBSERVATIONS.md OBS-056, OBS-068, OBS-069</t>
         </is>
       </c>
       <c r="D18" s="40" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="M18" s="40" t="inlineStr">
         <is>
-          <t>78/80 real, 2 structurally dead</t>
+          <t>477/481 = 99.17% real (up from 83.14% at 2026-09-06 freeze, 3 gap-hunt rounds 2026-09-20); 2 permanently structurally dead (fence.i, nop); 4 bins honestly open (see RISCVISACOV_STATUS.md, RISCVISACOV_INSTRUCTION_REFERENCE.md)</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="D14" s="40" t="inlineStr">
         <is>
-          <t>targeted single-kernel +ISACOV gap-hunt</t>
+          <t>targeted single-kernel +ISACOV gap-hunt (isacov_fill, 3 rounds)</t>
         </is>
       </c>
       <c r="E14" s="40" t="inlineStr">
@@ -4924,12 +4924,12 @@
       </c>
       <c r="G14" s="40" t="inlineStr">
         <is>
-          <t>78/80 real, 2 structurally dead (fence.i, unset-define coverpoint)</t>
+          <t>extends the standard model at its scalar boundary, does not replace it; per-instruction detail in riscvisacov/RISCVISACOV_INSTRUCTION_REFERENCE.md</t>
         </is>
       </c>
       <c r="H14" s="40" t="inlineStr">
         <is>
-          <t>78/80 = 97.5%</t>
+          <t>477/481 = 99.17% (99.57% weighted), up from 83.14% at the 2026-09-06 freeze</t>
         </is>
       </c>
     </row>
@@ -7140,11 +7140,31 @@
       </c>
     </row>
     <row r="14" ht="25.5" customHeight="1">
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>v1.1</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>Samuel Moussa</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>riscvISACOV L1 gap-hunt re-opened and taken from 83.14% (2026-09-06 freeze) to 99.17% (477/481 bins, 99.57% weighted) over 3 stimulus rounds, each re-verified byte-exact under LOCKSTEP before banking; new per-instruction reference doc (RISCVISACOV_INSTRUCTION_REFERENCE.md, all 80 covergroups); OBS-068 (branch/jal disassembly parsing bug) and OBS-069 (open lhu sign anomaly) found and disclosed; Coverage_Model_Reference.md stale-figure reconciled</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="25.5" customHeight="1">
       <c r="B15" s="16" t="n"/>

</xml_diff>